<commit_message>
Auto update metal rates
</commit_message>
<xml_diff>
--- a/metal_rates.xlsx
+++ b/metal_rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,79 +434,99 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Gold 24K 995</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Gold 24K 995GW</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Gold 22K</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Gold 18K</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Gold 14K</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Gold 9K</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
         <is>
           <t>Silver</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Silver Bar</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Platinum</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Source</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>17:58:45</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>14500</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>13174</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>11098</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>8592</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>227</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>230</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>7200</t>
+          <t>00:20:20</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>14500</v>
+      </c>
+      <c r="D2" t="n">
+        <v>14470</v>
+      </c>
+      <c r="E2" t="n">
+        <v>14290</v>
+      </c>
+      <c r="F2" t="n">
+        <v>13174</v>
+      </c>
+      <c r="G2" t="n">
+        <v>11098</v>
+      </c>
+      <c r="H2" t="n">
+        <v>8592</v>
+      </c>
+      <c r="I2" t="n">
+        <v>5728</v>
+      </c>
+      <c r="J2" t="n">
+        <v>227</v>
+      </c>
+      <c r="K2" t="n">
+        <v>230</v>
+      </c>
+      <c r="L2" t="n">
+        <v>7200</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>API</t>
         </is>
       </c>
     </row>

</xml_diff>